<commit_message>
Deploying to gh-pages from  @ 97cf749fd4c27d44e21332d00ff387afe0aab771 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_1-2-3.xlsx
+++ b/assets/excel/2026_1-2-3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9506499-64A9-4421-BDD4-2B0CE2D3F385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA5728CB-E639-491D-85FA-025817DA22FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{7A2C9C5F-6188-4B6C-9270-BAA72B6F2974}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{7A2C9C5F-6188-4B6C-9270-BAA72B6F2974}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -435,13 +435,13 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -463,9 +463,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -503,7 +503,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -609,7 +609,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -751,7 +751,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -794,50 +794,50 @@
       </c>
     </row>
     <row r="6" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17" t="s">
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="N6" s="17" t="s">
+      <c r="N6" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="17"/>
-      <c r="R6" s="17"/>
-      <c r="S6" s="17"/>
-      <c r="T6" s="17" t="s">
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="U6" s="17" t="s">
+      <c r="U6" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="V6" s="17"/>
-      <c r="W6" s="17"/>
-      <c r="X6" s="17"/>
-      <c r="Y6" s="17"/>
-      <c r="Z6" s="18"/>
+      <c r="V6" s="18"/>
+      <c r="W6" s="18"/>
+      <c r="X6" s="18"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="19"/>
     </row>
     <row r="7" spans="2:26" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="D7" s="19"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
       <c r="G7" s="3" t="s">
         <v>10</v>
       </c>
@@ -856,7 +856,7 @@
       <c r="L7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M7" s="17"/>
+      <c r="M7" s="18"/>
       <c r="N7" s="3" t="s">
         <v>10</v>
       </c>
@@ -875,7 +875,7 @@
       <c r="S7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="17"/>
+      <c r="T7" s="18"/>
       <c r="U7" s="3" t="s">
         <v>10</v>
       </c>
@@ -902,35 +902,35 @@
       <c r="C8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="19"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17" t="s">
+      <c r="D8" s="17"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17" t="s">
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
-      <c r="P8" s="17"/>
-      <c r="Q8" s="17"/>
-      <c r="R8" s="17"/>
-      <c r="S8" s="17"/>
-      <c r="T8" s="17" t="s">
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="18"/>
+      <c r="T8" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="U8" s="17"/>
-      <c r="V8" s="17"/>
-      <c r="W8" s="17"/>
-      <c r="X8" s="17"/>
-      <c r="Y8" s="17"/>
-      <c r="Z8" s="18"/>
+      <c r="U8" s="18"/>
+      <c r="V8" s="18"/>
+      <c r="W8" s="18"/>
+      <c r="X8" s="18"/>
+      <c r="Y8" s="18"/>
+      <c r="Z8" s="19"/>
     </row>
     <row r="9" spans="2:26" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C9" s="11">
@@ -84392,7 +84392,7 @@
         <v>122577</v>
       </c>
     </row>
-    <row r="1101" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="1101" spans="2:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1101" s="6" t="s">
         <v>23</v>
       </c>
@@ -84463,7 +84463,7 @@
         <v>4719</v>
       </c>
     </row>
-    <row r="1102" spans="2:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1102" spans="2:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1102" s="6" t="s">
         <v>24</v>
       </c>
@@ -84534,7 +84534,7 @@
         <v>3254</v>
       </c>
     </row>
-    <row r="1103" spans="2:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1103" spans="2:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1103" s="6" t="s">
         <v>25</v>
       </c>
@@ -84605,7 +84605,7 @@
         <v>3415</v>
       </c>
     </row>
-    <row r="1104" spans="2:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1104" spans="2:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1104" s="6" t="s">
         <v>26</v>
       </c>
@@ -84676,7 +84676,7 @@
         <v>2135</v>
       </c>
     </row>
-    <row r="1105" spans="4:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1105" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1105" s="6" t="s">
         <v>27</v>
       </c>
@@ -84747,7 +84747,7 @@
         <v>1898</v>
       </c>
     </row>
-    <row r="1106" spans="4:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1106" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1106" s="6" t="s">
         <v>28</v>
       </c>
@@ -84818,7 +84818,7 @@
         <v>1044</v>
       </c>
     </row>
-    <row r="1107" spans="4:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1107" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1107" s="6" t="s">
         <v>29</v>
       </c>
@@ -84889,7 +84889,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="1108" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1108" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1108" s="6" t="s">
         <v>30</v>
       </c>
@@ -84960,7 +84960,7 @@
         <v>2061</v>
       </c>
     </row>
-    <row r="1109" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1109" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1109" s="6" t="s">
         <v>31</v>
       </c>
@@ -85031,7 +85031,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="1110" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1110" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1110" s="6" t="s">
         <v>32</v>
       </c>
@@ -85102,7 +85102,7 @@
         <v>4856</v>
       </c>
     </row>
-    <row r="1111" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1111" spans="4:26" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1111" s="7" t="s">
         <v>33</v>
       </c>
@@ -85173,7 +85173,7 @@
         <v>26380</v>
       </c>
     </row>
-    <row r="1112" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1112" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1112" s="6" t="s">
         <v>34</v>
       </c>
@@ -85244,7 +85244,7 @@
         <v>30707</v>
       </c>
     </row>
-    <row r="1113" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1113" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1113" s="6" t="s">
         <v>35</v>
       </c>
@@ -85315,7 +85315,7 @@
         <v>19377</v>
       </c>
     </row>
-    <row r="1114" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1114" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1114" s="6" t="s">
         <v>36</v>
       </c>
@@ -85386,7 +85386,7 @@
         <v>11330</v>
       </c>
     </row>
-    <row r="1115" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1115" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1115" s="6" t="s">
         <v>37</v>
       </c>
@@ -85457,7 +85457,7 @@
         <v>2168</v>
       </c>
     </row>
-    <row r="1116" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1116" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1116" s="6" t="s">
         <v>38</v>
       </c>
@@ -85528,7 +85528,7 @@
         <v>3177</v>
       </c>
     </row>
-    <row r="1117" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1117" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1117" s="6" t="s">
         <v>39</v>
       </c>
@@ -85599,7 +85599,7 @@
         <v>3977</v>
       </c>
     </row>
-    <row r="1118" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1118" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1118" s="6" t="s">
         <v>40</v>
       </c>
@@ -85670,7 +85670,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="1119" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1119" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1119" s="6" t="s">
         <v>41</v>
       </c>
@@ -85741,7 +85741,7 @@
         <v>1528</v>
       </c>
     </row>
-    <row r="1120" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1120" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1120" s="6" t="s">
         <v>42</v>
       </c>
@@ -85812,7 +85812,7 @@
         <v>3047</v>
       </c>
     </row>
-    <row r="1121" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1121" spans="4:26" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1121" s="7" t="s">
         <v>43</v>
       </c>
@@ -85883,7 +85883,7 @@
         <v>45622</v>
       </c>
     </row>
-    <row r="1122" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1122" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1122" s="6" t="s">
         <v>44</v>
       </c>
@@ -85954,7 +85954,7 @@
         <v>2173</v>
       </c>
     </row>
-    <row r="1123" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1123" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1123" s="6" t="s">
         <v>45</v>
       </c>
@@ -86025,7 +86025,7 @@
         <v>2632</v>
       </c>
     </row>
-    <row r="1124" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1124" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1124" s="6" t="s">
         <v>46</v>
       </c>
@@ -86096,7 +86096,7 @@
         <v>3044</v>
       </c>
     </row>
-    <row r="1125" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1125" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1125" s="6" t="s">
         <v>47</v>
       </c>
@@ -86167,7 +86167,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="1126" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1126" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1126" s="6" t="s">
         <v>48</v>
       </c>
@@ -86238,7 +86238,7 @@
         <v>1536</v>
       </c>
     </row>
-    <row r="1127" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1127" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1127" s="6" t="s">
         <v>49</v>
       </c>
@@ -86309,7 +86309,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1128" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1128" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1128" s="6" t="s">
         <v>50</v>
       </c>
@@ -86380,7 +86380,7 @@
         <v>1456</v>
       </c>
     </row>
-    <row r="1129" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1129" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1129" s="6" t="s">
         <v>51</v>
       </c>
@@ -86451,7 +86451,7 @@
         <v>1491</v>
       </c>
     </row>
-    <row r="1130" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1130" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1130" s="6" t="s">
         <v>52</v>
       </c>
@@ -86522,7 +86522,7 @@
         <v>1958</v>
       </c>
     </row>
-    <row r="1131" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1131" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1131" s="6" t="s">
         <v>53</v>
       </c>
@@ -86593,7 +86593,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="1132" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1132" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1132" s="6" t="s">
         <v>54</v>
       </c>
@@ -86664,7 +86664,7 @@
         <v>1980</v>
       </c>
     </row>
-    <row r="1133" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1133" spans="4:26" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1133" s="7" t="s">
         <v>55</v>
       </c>
@@ -86735,7 +86735,7 @@
         <v>18287</v>
       </c>
     </row>
-    <row r="1134" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1134" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1134" s="6" t="s">
         <v>56</v>
       </c>
@@ -86806,7 +86806,7 @@
         <v>1944</v>
       </c>
     </row>
-    <row r="1135" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1135" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1135" s="6" t="s">
         <v>57</v>
       </c>
@@ -86877,7 +86877,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="1136" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1136" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1136" s="6" t="s">
         <v>58</v>
       </c>
@@ -86948,7 +86948,7 @@
         <v>1960</v>
       </c>
     </row>
-    <row r="1137" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1137" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1137" s="6" t="s">
         <v>59</v>
       </c>
@@ -87019,7 +87019,7 @@
         <v>3557</v>
       </c>
     </row>
-    <row r="1138" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1138" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1138" s="6" t="s">
         <v>60</v>
       </c>
@@ -87090,7 +87090,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="1139" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1139" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1139" s="6" t="s">
         <v>61</v>
       </c>
@@ -87161,7 +87161,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="1140" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1140" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1140" s="6" t="s">
         <v>62</v>
       </c>
@@ -87232,7 +87232,7 @@
         <v>1234</v>
       </c>
     </row>
-    <row r="1141" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1141" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1141" s="6" t="s">
         <v>63</v>
       </c>
@@ -87303,7 +87303,7 @@
         <v>1124</v>
       </c>
     </row>
-    <row r="1142" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1142" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1142" s="6" t="s">
         <v>64</v>
       </c>
@@ -87374,7 +87374,7 @@
         <v>2300</v>
       </c>
     </row>
-    <row r="1143" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1143" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1143" s="6" t="s">
         <v>65</v>
       </c>
@@ -87445,7 +87445,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="1144" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1144" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1144" s="6" t="s">
         <v>66</v>
       </c>
@@ -87516,7 +87516,7 @@
         <v>2770</v>
       </c>
     </row>
-    <row r="1145" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1145" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1145" s="6" t="s">
         <v>67</v>
       </c>
@@ -87587,7 +87587,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="1146" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1146" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1146" s="6" t="s">
         <v>68</v>
       </c>
@@ -87658,7 +87658,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="1147" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1147" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1147" s="6" t="s">
         <v>69</v>
       </c>
@@ -87729,7 +87729,7 @@
         <v>4216</v>
       </c>
     </row>
-    <row r="1148" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1148" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1148" s="6" t="s">
         <v>70</v>
       </c>
@@ -87800,7 +87800,7 @@
         <v>1814</v>
       </c>
     </row>
-    <row r="1149" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1149" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1149" s="6" t="s">
         <v>71</v>
       </c>
@@ -87871,7 +87871,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="1150" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1150" spans="4:26" s="6" customFormat="1" ht="8.25" x14ac:dyDescent="0.15">
       <c r="D1150" s="6" t="s">
         <v>72</v>
       </c>
@@ -87942,7 +87942,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="1151" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1151" spans="4:26" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1151" s="7" t="s">
         <v>73</v>
       </c>
@@ -88013,7 +88013,7 @@
         <v>28042</v>
       </c>
     </row>
-    <row r="1152" spans="4:26" x14ac:dyDescent="0.25">
+    <row r="1152" spans="4:26" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1152" s="7" t="s">
         <v>74</v>
       </c>
@@ -88084,44 +88084,45 @@
         <v>118331</v>
       </c>
     </row>
-    <row r="1154" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="1154" spans="4:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1154" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="1156" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="1155" spans="4:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1156" spans="4:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1156" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="1157" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="1157" spans="4:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1157" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="1158" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="1158" spans="4:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1158" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="1159" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="1159" spans="4:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1159" s="10" t="s">
         <v>22</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:L6"/>
-    <mergeCell ref="M6:M7"/>
     <mergeCell ref="T6:T7"/>
     <mergeCell ref="U6:Z6"/>
     <mergeCell ref="F8:L8"/>
     <mergeCell ref="M8:S8"/>
     <mergeCell ref="T8:Z8"/>
     <mergeCell ref="N6:S6"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:L6"/>
+    <mergeCell ref="M6:M7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D1159" r:id="rId1" xr:uid="{A02DF72A-83D0-4B18-BE63-0CD0144D427E}"/>

</xml_diff>